<commit_message>
25th Arpil File Update
</commit_message>
<xml_diff>
--- a/Compititor's_Price/Celotex_Prices/Celotex_Prices_25-04-2025.xlsx
+++ b/Compititor's_Price/Celotex_Prices/Celotex_Prices_25-04-2025.xlsx
@@ -2,15 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -26,7 +25,9 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,10 +47,19 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -62,7 +72,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -152,6 +162,11 @@
         <t>Previous Price: £11.17</t>
       </text>
     </comment>
+    <comment ref="E2" authorId="0" shapeId="0">
+      <text>
+        <t>Previous Price: £11.17</t>
+      </text>
+    </comment>
     <comment ref="F2" authorId="0" shapeId="0">
       <text>
         <t>Previous Price: £11.50</t>
@@ -187,6 +202,11 @@
         <t>Previous Price: £13.30</t>
       </text>
     </comment>
+    <comment ref="E3" authorId="0" shapeId="0">
+      <text>
+        <t>Previous Price: £13.30</t>
+      </text>
+    </comment>
     <comment ref="F3" authorId="0" shapeId="0">
       <text>
         <t>Previous Price: £13.50</t>
@@ -222,6 +242,11 @@
         <t>Previous Price: £15.95</t>
       </text>
     </comment>
+    <comment ref="E4" authorId="0" shapeId="0">
+      <text>
+        <t>Previous Price: £15.95</t>
+      </text>
+    </comment>
     <comment ref="F4" authorId="0" shapeId="0">
       <text>
         <t>Previous Price: £15.95</t>
@@ -257,6 +282,11 @@
         <t>Previous Price: £16.95</t>
       </text>
     </comment>
+    <comment ref="E5" authorId="0" shapeId="0">
+      <text>
+        <t>Previous Price: £16.95</t>
+      </text>
+    </comment>
     <comment ref="F5" authorId="0" shapeId="0">
       <text>
         <t>Previous Price: £16.95</t>
@@ -292,6 +322,11 @@
         <t>Previous Price: £21.50</t>
       </text>
     </comment>
+    <comment ref="E6" authorId="0" shapeId="0">
+      <text>
+        <t>Previous Price: £21.50</t>
+      </text>
+    </comment>
     <comment ref="F6" authorId="0" shapeId="0">
       <text>
         <t>Previous Price: £21.50</t>
@@ -327,6 +362,11 @@
         <t>Previous Price: £23.95</t>
       </text>
     </comment>
+    <comment ref="E7" authorId="0" shapeId="0">
+      <text>
+        <t>Previous Price: £23.95</t>
+      </text>
+    </comment>
     <comment ref="F7" authorId="0" shapeId="0">
       <text>
         <t>Previous Price: £23.95</t>
@@ -362,6 +402,11 @@
         <t>Previous Price: £23.50</t>
       </text>
     </comment>
+    <comment ref="E8" authorId="0" shapeId="0">
+      <text>
+        <t>Previous Price: £23.50</t>
+      </text>
+    </comment>
     <comment ref="F8" authorId="0" shapeId="0">
       <text>
         <t>Previous Price: £23.50</t>
@@ -397,6 +442,11 @@
         <t>Previous Price: £26.95</t>
       </text>
     </comment>
+    <comment ref="E9" authorId="0" shapeId="0">
+      <text>
+        <t>Previous Price: £26.95</t>
+      </text>
+    </comment>
     <comment ref="F9" authorId="0" shapeId="0">
       <text>
         <t>Previous Price: £26.95</t>
@@ -432,6 +482,11 @@
         <t>Previous Price: £28.95</t>
       </text>
     </comment>
+    <comment ref="E10" authorId="0" shapeId="0">
+      <text>
+        <t>Previous Price: £28.95</t>
+      </text>
+    </comment>
     <comment ref="F10" authorId="0" shapeId="0">
       <text>
         <t>Previous Price: £28.95</t>
@@ -467,6 +522,11 @@
         <t>Previous Price: £28.95</t>
       </text>
     </comment>
+    <comment ref="E11" authorId="0" shapeId="0">
+      <text>
+        <t>Previous Price: £28.95</t>
+      </text>
+    </comment>
     <comment ref="F11" authorId="0" shapeId="0">
       <text>
         <t>Previous Price: £28.95</t>
@@ -502,6 +562,11 @@
         <t>Previous Price: £37.95</t>
       </text>
     </comment>
+    <comment ref="E12" authorId="0" shapeId="0">
+      <text>
+        <t>Previous Price: £37.95</t>
+      </text>
+    </comment>
     <comment ref="F12" authorId="0" shapeId="0">
       <text>
         <t>Previous Price: £37.95</t>
@@ -537,6 +602,11 @@
         <t>Previous Price: £34.95</t>
       </text>
     </comment>
+    <comment ref="E13" authorId="0" shapeId="0">
+      <text>
+        <t>Previous Price: £34.95</t>
+      </text>
+    </comment>
     <comment ref="F13" authorId="0" shapeId="0">
       <text>
         <t>Previous Price: £34.95</t>
@@ -572,6 +642,11 @@
         <t>Previous Price: £42.50</t>
       </text>
     </comment>
+    <comment ref="E14" authorId="0" shapeId="0">
+      <text>
+        <t>Previous Price: £42.50</t>
+      </text>
+    </comment>
     <comment ref="F14" authorId="0" shapeId="0">
       <text>
         <t>Previous Price: £42.50</t>
@@ -642,6 +717,11 @@
         <t>Previous Price: £44.95</t>
       </text>
     </comment>
+    <comment ref="E16" authorId="0" shapeId="0">
+      <text>
+        <t>Previous Price: £44.95</t>
+      </text>
+    </comment>
     <comment ref="F16" authorId="0" shapeId="0">
       <text>
         <t>Previous Price: £44.95</t>
@@ -677,6 +757,11 @@
         <t>Previous Price: £729.95</t>
       </text>
     </comment>
+    <comment ref="E17" authorId="0" shapeId="0">
+      <text>
+        <t>Previous Price: £729.95</t>
+      </text>
+    </comment>
     <comment ref="F17" authorId="0" shapeId="0">
       <text>
         <t>Previous Price: £729.95</t>
@@ -712,6 +797,11 @@
         <t>Previous Price: £935.40</t>
       </text>
     </comment>
+    <comment ref="E18" authorId="0" shapeId="0">
+      <text>
+        <t>Previous Price: £935.40</t>
+      </text>
+    </comment>
     <comment ref="F18" authorId="0" shapeId="0">
       <text>
         <t>Previous Price: £934.95</t>
@@ -742,6 +832,11 @@
         <t>Previous Price: £32.75</t>
       </text>
     </comment>
+    <comment ref="E19" authorId="0" shapeId="0">
+      <text>
+        <t>Previous Price: £32.75</t>
+      </text>
+    </comment>
     <comment ref="F19" authorId="0" shapeId="0">
       <text>
         <t>Previous Price: £35.50</t>
@@ -772,6 +867,11 @@
         <t>Previous Price: £38.75</t>
       </text>
     </comment>
+    <comment ref="E20" authorId="0" shapeId="0">
+      <text>
+        <t>Previous Price: £38.75</t>
+      </text>
+    </comment>
     <comment ref="F20" authorId="0" shapeId="0">
       <text>
         <t>Previous Price: £44.50</t>
@@ -802,6 +902,11 @@
         <t>Previous Price: £43.60</t>
       </text>
     </comment>
+    <comment ref="E21" authorId="0" shapeId="0">
+      <text>
+        <t>Previous Price: £43.60</t>
+      </text>
+    </comment>
     <comment ref="F21" authorId="0" shapeId="0">
       <text>
         <t>Previous Price: £46.95</t>
@@ -832,6 +937,11 @@
         <t>Previous Price: £48.65</t>
       </text>
     </comment>
+    <comment ref="E22" authorId="0" shapeId="0">
+      <text>
+        <t>Previous Price: £48.65</t>
+      </text>
+    </comment>
     <comment ref="F22" authorId="0" shapeId="0">
       <text>
         <t>Previous Price: £52.50</t>
@@ -862,6 +972,11 @@
         <t>Previous Price: £45.50</t>
       </text>
     </comment>
+    <comment ref="E23" authorId="0" shapeId="0">
+      <text>
+        <t>Previous Price: £45.50</t>
+      </text>
+    </comment>
     <comment ref="F23" authorId="0" shapeId="0">
       <text>
         <t>Previous Price: £45.50</t>
@@ -887,6 +1002,11 @@
         <t>Previous Price: £43.80</t>
       </text>
     </comment>
+    <comment ref="E24" authorId="0" shapeId="0">
+      <text>
+        <t>Previous Price: £43.80</t>
+      </text>
+    </comment>
     <comment ref="F24" authorId="0" shapeId="0">
       <text>
         <t>Previous Price: £43.95</t>
@@ -912,6 +1032,11 @@
         <t>Previous Price: £924.50</t>
       </text>
     </comment>
+    <comment ref="E25" authorId="0" shapeId="0">
+      <text>
+        <t>Previous Price: £924.50</t>
+      </text>
+    </comment>
     <comment ref="P25" authorId="0" shapeId="0">
       <text>
         <t>Previous Price: £1189.28</t>
@@ -927,6 +1052,11 @@
         <t>Previous Price: £44.65</t>
       </text>
     </comment>
+    <comment ref="E26" authorId="0" shapeId="0">
+      <text>
+        <t>Previous Price: £44.65</t>
+      </text>
+    </comment>
     <comment ref="F26" authorId="0" shapeId="0">
       <text>
         <t>Previous Price: £44.95</t>
@@ -937,6 +1067,11 @@
         <t>Previous Price: £29.59</t>
       </text>
     </comment>
+    <comment ref="J26" authorId="0" shapeId="0">
+      <text>
+        <t>Previous Price: £12.41</t>
+      </text>
+    </comment>
     <comment ref="N26" authorId="0" shapeId="0">
       <text>
         <t>Previous Price: £43.78</t>
@@ -957,6 +1092,11 @@
         <t>Previous Price: £1,163.00</t>
       </text>
     </comment>
+    <comment ref="E27" authorId="0" shapeId="0">
+      <text>
+        <t>Previous Price: £1,165.00</t>
+      </text>
+    </comment>
     <comment ref="F27" authorId="0" shapeId="0">
       <text>
         <t>Previous Price: £1,164.95</t>
@@ -982,6 +1122,11 @@
         <t>Previous Price: £1,268.00</t>
       </text>
     </comment>
+    <comment ref="E28" authorId="0" shapeId="0">
+      <text>
+        <t>Previous Price: £1,268.00</t>
+      </text>
+    </comment>
     <comment ref="F28" authorId="0" shapeId="0">
       <text>
         <t>Previous Price: £1,274.95</t>
@@ -1003,6 +1148,11 @@
       </text>
     </comment>
     <comment ref="D29" authorId="0" shapeId="0">
+      <text>
+        <t>Previous Price: £1,210.00</t>
+      </text>
+    </comment>
+    <comment ref="E29" authorId="0" shapeId="0">
       <text>
         <t>Previous Price: £1,210.00</t>
       </text>
@@ -1438,7 +1588,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>£11.17</t>
+          <t>£12.41</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1535,7 +1685,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>£13.30</t>
+          <t>£14.78</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1632,7 +1782,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>£15.95</t>
+          <t>£17.72</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1729,7 +1879,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>£16.95</t>
+          <t>£18.83</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1826,7 +1976,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>£21.50</t>
+          <t>£23.89</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1923,7 +2073,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>£23.95</t>
+          <t>£26.61</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -2020,7 +2170,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>£23.50</t>
+          <t>£26.11</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -2117,7 +2267,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>£26.95</t>
+          <t>£29.94</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -2214,7 +2364,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>£28.95</t>
+          <t>£32.17</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -2311,7 +2461,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>£28.95</t>
+          <t>£32.17</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -2408,7 +2558,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>£37.95</t>
+          <t>£42.17</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -2505,7 +2655,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>£34.95</t>
+          <t>£38.83</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -2602,7 +2752,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>£42.50</t>
+          <t>£47.22</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -2796,7 +2946,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>£44.95</t>
+          <t>£49.94</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2893,7 +3043,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>£729.95</t>
+          <t>£811.06</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2990,7 +3140,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>£935.40</t>
+          <t>£1,039.33</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -3087,7 +3237,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>£32.75</t>
+          <t>£36.39</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -3184,7 +3334,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>£38.75</t>
+          <t>£43.06</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -3281,7 +3431,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>£43.60</t>
+          <t>£48.44</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -3378,7 +3528,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>£48.65</t>
+          <t>£54.06</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -3475,7 +3625,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>£45.50</t>
+          <t>£50.56</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -3572,7 +3722,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>£43.80</t>
+          <t>£48.68</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -3669,7 +3819,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>£924.50</t>
+          <t>£1,027.22</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3766,7 +3916,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>£44.65</t>
+          <t>£49.61</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3776,7 +3926,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>£29.99</t>
+          <t>£52.95</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -3791,7 +3941,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>£12.41</t>
+          <t>£74.46</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -3863,7 +4013,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>£1,165.00</t>
+          <t>£1,292.22</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3960,7 +4110,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>£1,268.00</t>
+          <t>£1,408.89</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -4057,7 +4207,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>£1,210.00</t>
+          <t>£1,344.44</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">

</xml_diff>